<commit_message>
Add Workday, SmartRecruiters and Ashby scrapers; refresh seed list with search and location options
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015uMR1iyRxzVzihGimcJPB4
</commit_message>
<xml_diff>
--- a/docs/seed-sources/jobHunt_sources.xlsx
+++ b/docs/seed-sources/jobHunt_sources.xlsx
@@ -1595,7 +1595,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/aiprise</t>
+          <t>https://jobs.ashbyhq.com/aiprise?location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1626,7 +1626,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/certifyos</t>
+          <t>https://jobs.ashbyhq.com/certifyos?location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1657,7 +1657,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/bolna</t>
+          <t>https://jobs.ashbyhq.com/bolna?location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1688,7 +1688,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/savvymoney</t>
+          <t>https://jobs.ashbyhq.com/savvymoney?location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1723,7 +1723,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/bjakcareer</t>
+          <t>https://jobs.ashbyhq.com/bjakcareer?location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1754,7 +1754,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/uipath</t>
+          <t>https://jobs.ashbyhq.com/uipath?location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1785,7 +1785,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/tekion</t>
+          <t>https://jobs.ashbyhq.com/tekion?location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1816,7 +1816,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/firstwork</t>
+          <t>https://jobs.ashbyhq.com/firstwork?location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/furtherai</t>
+          <t>https://jobs.ashbyhq.com/furtherai?location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1878,7 +1878,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/cartesia</t>
+          <t>https://jobs.ashbyhq.com/cartesia?location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1909,7 +1909,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers</t>
+          <t>https://mastercard.wd1.myworkdayjobs.com/CorporateCareers?q=java&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1940,7 +1940,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>https://paypal.wd1.myworkdayjobs.com/jobs</t>
+          <t>https://paypal.wd1.myworkdayjobs.com/jobs?q=java&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1971,7 +1971,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>https://statestreet.wd1.myworkdayjobs.com/Global</t>
+          <t>https://statestreet.wd1.myworkdayjobs.com/Global?q=java&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2002,7 +2002,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>https://wf.wd1.myworkdayjobs.com/WellsFargoJobs</t>
+          <t>https://wf.wd1.myworkdayjobs.com/WellsFargoJobs?q=java&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2033,7 +2033,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>https://ms.wd5.myworkdayjobs.com/External</t>
+          <t>https://ms.wd5.myworkdayjobs.com/External?q=java&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2064,7 +2064,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>https://worldpay.wd5.myworkdayjobs.com/Worldpay_External_Careers_Site</t>
+          <t>https://worldpay.wd5.myworkdayjobs.com/Worldpay_External_Careers_Site?q=java&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2095,7 +2095,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>https://jda.wd5.myworkdayjobs.com/JDA_Careers</t>
+          <t>https://jda.wd5.myworkdayjobs.com/JDA_Careers?q=java&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2126,7 +2126,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>https://redhat.wd5.myworkdayjobs.com/Jobs</t>
+          <t>https://redhat.wd5.myworkdayjobs.com/Jobs?q=software+engineer&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2157,7 +2157,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>https://reliaquest.wd5.myworkdayjobs.com/ReliaQuest_Careers</t>
+          <t>https://reliaquest.wd5.myworkdayjobs.com/ReliaQuest_Careers?q=software+engineer&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2188,7 +2188,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://cdk.wd1.myworkdayjobs.com/CDK</t>
+          <t>https://cdk.wd1.myworkdayjobs.com/CDK?q=java&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2219,7 +2219,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>https://web.wd1.myworkdayjobs.com/ExternalCareerSite</t>
+          <t>https://web.wd1.myworkdayjobs.com/ExternalCareerSite?q=java&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2250,7 +2250,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>https://spgi.wd5.myworkdayjobs.com/spgi_internal</t>
+          <t>https://spgi.wd5.myworkdayjobs.com/spgi_internal?q=java&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2281,7 +2281,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>https://gartner.wd5.myworkdayjobs.com/EXT</t>
+          <t>https://gartner.wd5.myworkdayjobs.com/EXT?q=java&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2312,7 +2312,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>https://mavenir.wd1.myworkdayjobs.com/Mavenir_Careers</t>
+          <t>https://mavenir.wd1.myworkdayjobs.com/Mavenir_Careers?q=java&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2343,7 +2343,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>https://motorolasolutions.wd5.myworkdayjobs.com/Careers</t>
+          <t>https://motorolasolutions.wd5.myworkdayjobs.com/Careers?q=java&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2374,7 +2374,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>https://gevernova.wd5.myworkdayjobs.com/Vernova_ExternalSite</t>
+          <t>https://gevernova.wd5.myworkdayjobs.com/Vernova_ExternalSite?q=java&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2405,7 +2405,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>https://hitachi.wd1.myworkdayjobs.com/hitachi</t>
+          <t>https://hitachi.wd1.myworkdayjobs.com/hitachi?q=java&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2436,7 +2436,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>https://hpe.wd5.myworkdayjobs.com/ACJobSite</t>
+          <t>https://hpe.wd5.myworkdayjobs.com/ACJobSite?q=software+engineer&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2467,7 +2467,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>https://nxp.wd3.myworkdayjobs.com/careers</t>
+          <t>https://nxp.wd3.myworkdayjobs.com/careers?q=embedded&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2498,7 +2498,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>https://sensata.wd1.myworkdayjobs.com/Sensata-Careers</t>
+          <t>https://sensata.wd1.myworkdayjobs.com/Sensata-Careers?q=embedded&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2529,7 +2529,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>https://hp.wd5.myworkdayjobs.com/ExternalCareerSite</t>
+          <t>https://hp.wd5.myworkdayjobs.com/ExternalCareerSite?q=embedded&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2560,7 +2560,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>https://careers.smartrecruiters.com/servicenow?search=India</t>
+          <t>https://careers.smartrecruiters.com/servicenow?search=India&amp;location=India</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2591,7 +2591,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>https://careers.smartrecruiters.com/Visa</t>
+          <t>https://careers.smartrecruiters.com/Visa?search=India&amp;location=India</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2622,7 +2622,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>https://careers.smartrecruiters.com/Experian</t>
+          <t>https://careers.smartrecruiters.com/Experian?search=India&amp;location=India</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2653,7 +2653,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>https://careers.smartrecruiters.com/Zscaler</t>
+          <t>https://careers.smartrecruiters.com/Zscaler?search=India&amp;location=India</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2684,7 +2684,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>https://careers.smartrecruiters.com/WesternDigital</t>
+          <t>https://careers.smartrecruiters.com/WesternDigital?search=embedded&amp;location=India</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2715,7 +2715,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>https://careers.smartrecruiters.com/NECSWS</t>
+          <t>https://careers.smartrecruiters.com/NECSWS?search=java&amp;location=India</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -4358,7 +4358,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>https://nvidia.wd5.myworkdayjobs.com/NVIDIAExternalCareerSite</t>
+          <t>https://nvidia.wd5.myworkdayjobs.com/NVIDIAExternalCareerSite?q=embedded&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -4389,7 +4389,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>https://cadence.wd1.myworkdayjobs.com/External_Careers</t>
+          <t>https://cadence.wd1.myworkdayjobs.com/External_Careers?q=software+engineer&amp;location=India|Bengaluru|Bangalore|Hyderabad|Pune|Chennai|Mumbai|Gurugram|Gurgaon|Noida|Delhi</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -5542,7 +5542,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/syndica</t>
+          <t>https://jobs.ashbyhq.com/syndica?location=Dubai|Abu Dhabi|Sharjah|United Arab Emirates</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -5573,7 +5573,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://careers.smartrecruiters.com/DeliveryHero?search=Dubai</t>
+          <t>https://careers.smartrecruiters.com/DeliveryHero?search=Dubai&amp;location=Dubai|Abu Dhabi|Sharjah|United Arab Emirates</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -5604,7 +5604,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>https://careers.smartrecruiters.com/EtihadAirways5</t>
+          <t>https://careers.smartrecruiters.com/EtihadAirways5?search=United Arab Emirates&amp;location=Dubai|Abu Dhabi|Sharjah|United Arab Emirates</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -5635,7 +5635,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://careers.smartrecruiters.com/masdar</t>
+          <t>https://careers.smartrecruiters.com/masdar?search=United Arab Emirates&amp;location=Dubai|Abu Dhabi|Sharjah|United Arab Emirates</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -5666,7 +5666,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://careers.smartrecruiters.com/VAMS</t>
+          <t>https://careers.smartrecruiters.com/VAMS?search=United Arab Emirates&amp;location=Dubai|Abu Dhabi|Sharjah|United Arab Emirates</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -5697,7 +5697,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://careers.smartrecruiters.com/GhobashGroup</t>
+          <t>https://careers.smartrecruiters.com/GhobashGroup?search=United Arab Emirates&amp;location=Dubai|Abu Dhabi|Sharjah|United Arab Emirates</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">

</xml_diff>